<commit_message>
scan: seg8 2026-06-13 02:32 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq0_2026-06-12.xlsx
+++ b/output/full_scan/batch_seq0_2026-06-12.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>60.43324360906292</v>
+        <v>60.43324363652594</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>20.13825374732117</v>
+        <v>20.13825387069624</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>2.886606580279949</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>0.0533677870805422</v>
+        <v>0.0533677867535657</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -591,7 +591,7 @@
         <v/>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1067.16591985028</v>
+        <v>1082.16591985028</v>
       </c>
       <c r="E3" s="2" t="n">
         <v>22.45</v>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>70.94833636060329</v>
+        <v>70.9483363561596</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>41.35047776092387</v>
+        <v>41.35047773330003</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>2.216591985028026</v>
@@ -644,7 +644,7 @@
         <v/>
       </c>
       <c r="D4" s="2" t="n">
-        <v>1051.701874271119</v>
+        <v>1066.701874271119</v>
       </c>
       <c r="E4" s="2" t="n">
         <v>1475</v>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>58.91166499103494</v>
+        <v>58.91166497074728</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>27.66602479767439</v>
+        <v>27.66602480148545</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>1.170187427111906</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>-4.18646013239794</v>
+        <v>-4.186460131348596</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -686,21 +686,21 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>8112</v>
+        <v>8071</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>至上</t>
+          <t>能率網通</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
         <v/>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1027.453961803481</v>
+        <v>1027.78878647842</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>98.8</v>
+        <v>24.5</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -711,16 +711,16 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>64.1376352997392</v>
+        <v>65.23606995227618</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>24.03094808192049</v>
+        <v>39.52024715946621</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>1.74539618034815</v>
+        <v>2.778878647842028</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
         <v>0</v>
@@ -729,31 +729,31 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>0.7137544821635511</v>
+        <v>0.1969434675587635</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>8071</v>
+        <v>8112</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>能率網通</t>
+          <t>至上</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
         <v/>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1012.78878647842</v>
+        <v>1027.453961803481</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>24.5</v>
+        <v>98.8</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -764,16 +764,16 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>65.23606991528501</v>
+        <v>64.1376352997392</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>39.52024686027855</v>
+        <v>24.03094809190733</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>2.778878647842028</v>
+        <v>1.74539618034815</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L6" s="2" t="n">
         <v>0</v>
@@ -782,11 +782,11 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.1969434676923231</v>
+        <v>0.7137544819918502</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>62.79058500963205</v>
+        <v>62.79058504578</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>42.6408218288347</v>
+        <v>42.64082189631656</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>0.7414940604642128</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>-1.052309844234455</v>
+        <v>-1.052309844730509</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>63.55826787810334</v>
+        <v>63.55826826804881</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>23.64838917167713</v>
+        <v>23.64838925115862</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>1.766287510804795</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.1134262024447923</v>
+        <v>0.1134262022539954</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -909,7 +909,7 @@
         <v/>
       </c>
       <c r="D9" s="2" t="n">
-        <v>933.7616093083778</v>
+        <v>948.7616093083778</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>74.2</v>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>67.6921244462241</v>
+        <v>67.69212444941051</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>53.307027538113</v>
+        <v>53.30702769583197</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>0.8761609308377896</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.1601731967699287</v>
+        <v>0.1601731966936066</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -951,21 +951,21 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>8150</v>
+        <v>8163</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>南茂</t>
+          <t>達方</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
         <v/>
       </c>
       <c r="D10" s="2" t="n">
-        <v>930.8062684114814</v>
+        <v>942.7250289589496</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>97</v>
+        <v>42.85</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -976,49 +976,49 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>55.29989085496246</v>
+        <v>71.89806568354433</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>26.97825100891568</v>
+        <v>51.23135388854853</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>1.580626841148143</v>
+        <v>0.7725028958949451</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M10" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>-0.8834725196737576</v>
+        <v>0.1584687285755599</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, kd_golden_cross, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>8163</v>
+        <v>8150</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>達方</t>
+          <t>南茂</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
         <v/>
       </c>
       <c r="D11" s="2" t="n">
-        <v>927.7250289589496</v>
+        <v>930.8062684114814</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>42.85</v>
+        <v>97</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -1029,29 +1029,29 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>71.8980656447599</v>
+        <v>55.29989085807532</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>51.23135380420713</v>
+        <v>26.97825110653702</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>0.7725028958949451</v>
+        <v>1.580626841148143</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M11" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>0.1584687286709525</v>
+        <v>-0.883472519759616</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, kd_golden_cross, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>49.32658880510866</v>
+        <v>49.32658883754755</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>29.01493882452818</v>
+        <v>29.01493909848728</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>0.2508338718981917</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>-0.775368506315284</v>
+        <v>-0.7753685065442468</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1121,7 +1121,7 @@
         <v/>
       </c>
       <c r="D13" s="2" t="n">
-        <v>904.9252398380844</v>
+        <v>919.9252398380844</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>81.2</v>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>71.60011411070772</v>
+        <v>71.60011409965358</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>26.57582764550663</v>
+        <v>26.57582773984316</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>1.492523983808433</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>0.5327079460052055</v>
+        <v>0.5327079457380843</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1174,7 +1174,7 @@
         <v/>
       </c>
       <c r="D14" s="2" t="n">
-        <v>881.3015609005275</v>
+        <v>896.3015609005275</v>
       </c>
       <c r="E14" s="2" t="n">
         <v>19.65</v>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>77.40455511057596</v>
+        <v>77.40455522469297</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>35.94795979384654</v>
+        <v>35.94795991481855</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>2.130156090052749</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0.554921634014657</v>
+        <v>0.5549216338906432</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1227,7 +1227,7 @@
         <v/>
       </c>
       <c r="D15" s="2" t="n">
-        <v>859.9131524693986</v>
+        <v>874.9131524693986</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>348.5</v>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>62.46196038904545</v>
+        <v>62.46196044675006</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>21.9576324607627</v>
+        <v>21.95763246104672</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>0.4913152469398622</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>4.345390601163915</v>
+        <v>4.345390599732914</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1280,7 +1280,7 @@
         <v/>
       </c>
       <c r="D16" s="2" t="n">
-        <v>849.4829190961506</v>
+        <v>864.4829190961506</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>73.40000000000001</v>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>68.79161740096004</v>
+        <v>68.79161762824972</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>29.81811815196233</v>
+        <v>29.81811816545352</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>1.448291909615061</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0.3992496618341858</v>
+        <v>0.3992496611664031</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1322,21 +1322,21 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>8088</v>
+        <v>8121</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>品安</t>
+          <t>越峰</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
         <v/>
       </c>
       <c r="D17" s="2" t="n">
-        <v>841.1278246466454</v>
+        <v>853.7429718093272</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>61.4</v>
+        <v>44.4</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1347,16 +1347,16 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>55.28390423942511</v>
+        <v>65.71436039739331</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>23.79892964669937</v>
+        <v>43.71457495655156</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>0.612782464664544</v>
+        <v>0.8742971809327201</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L17" s="2" t="n">
         <v>0</v>
@@ -1365,31 +1365,31 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>-0.484341867273949</v>
+        <v>0.1022642457869258</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>8121</v>
+        <v>8088</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>越峰</t>
+          <t>品安</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
         <v/>
       </c>
       <c r="D18" s="2" t="n">
-        <v>838.7429718093272</v>
+        <v>841.1278246466454</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>44.4</v>
+        <v>61.4</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -1400,16 +1400,16 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>65.71436037404371</v>
+        <v>55.28390419864871</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>43.71457482905752</v>
+        <v>23.79892952605989</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>0.8742971809327201</v>
+        <v>0.612782464664544</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L18" s="2" t="n">
         <v>0</v>
@@ -1418,31 +1418,31 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>0.1022642459014027</v>
+        <v>-0.4843418667588055</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>8091</v>
+        <v>9136</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>翔名</t>
+          <t>巨騰-DR</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
         <v/>
       </c>
       <c r="D19" s="2" t="n">
-        <v>819.6732143125921</v>
+        <v>824.536910466572</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>241.5</v>
+        <v>17.35</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -1453,16 +1453,16 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>52.46226557882514</v>
+        <v>72.09003396534519</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>35.17565438411553</v>
+        <v>53.72399501641328</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>0.4673214312592068</v>
+        <v>1.453691046657196</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L19" s="2" t="n">
         <v>0</v>
@@ -1471,31 +1471,31 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>-5.245162265558067</v>
+        <v>0.3037952778632906</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, stronger_than_market, kd_golden_cross, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>9136</v>
+        <v>8091</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>巨騰-DR</t>
+          <t>翔名</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
         <v/>
       </c>
       <c r="D20" s="2" t="n">
-        <v>809.536910466572</v>
+        <v>819.6732143125921</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>17.35</v>
+        <v>241.5</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -1506,16 +1506,16 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>72.09003396983857</v>
+        <v>52.46226558177653</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>53.72399483117764</v>
+        <v>35.17565434093008</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>1.453691046657196</v>
+        <v>0.4673214312592068</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L20" s="2" t="n">
         <v>0</v>
@@ -1524,11 +1524,11 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0.3037952778270383</v>
+        <v>-5.245162265653468</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, stronger_than_market, kd_golden_cross, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -1545,7 +1545,7 @@
         <v/>
       </c>
       <c r="D21" s="2" t="n">
-        <v>803.7038377986966</v>
+        <v>818.7038377986966</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>82</v>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>57.08088765052366</v>
+        <v>57.08088756223188</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>21.55704188355697</v>
+        <v>21.55704190702665</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>2.37038377986966</v>
@@ -1598,7 +1598,7 @@
         <v/>
       </c>
       <c r="D22" s="2" t="n">
-        <v>792.2676332864226</v>
+        <v>807.2676332864226</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>53.6</v>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>67.94433352661559</v>
+        <v>67.94433354027029</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>26.84594047354009</v>
+        <v>26.84594057998677</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>3.226763328642256</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0.79274756863009</v>
+        <v>0.7927475685633087</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1640,21 +1640,21 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>8131</v>
+        <v>9910</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>福懋科</t>
+          <t>豐泰</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
         <v/>
       </c>
       <c r="D23" s="2" t="n">
-        <v>783.2554826840769</v>
+        <v>787.0901057180197</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>72</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
@@ -1665,16 +1665,16 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>56.03963651110419</v>
+        <v>68.02413660295505</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>14.32999462627285</v>
+        <v>32.06842880692204</v>
       </c>
       <c r="J23" s="2" t="n">
-        <v>0.8255482684076917</v>
+        <v>1.209010571801963</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L23" s="2" t="n">
         <v>0</v>
@@ -1683,31 +1683,31 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>-0.1626670062342454</v>
+        <v>2.650257112030566</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>9910</v>
+        <v>8131</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>豐泰</t>
+          <t>福懋科</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>772.0901057180197</v>
+        <v>783.2554826840769</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>91.90000000000001</v>
+        <v>72</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -1718,16 +1718,16 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>68.02413644010271</v>
+        <v>56.03963651110419</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>32.06842879811308</v>
+        <v>14.32999466961948</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>1.209010571801963</v>
+        <v>0.8255482684076917</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L24" s="2" t="n">
         <v>0</v>
@@ -1736,31 +1736,31 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>2.650257113175334</v>
+        <v>-0.1626670062819537</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>8093</v>
+        <v>8472</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>保銳</t>
+          <t>夠麻吉</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>769.5892506265369</v>
+        <v>775.6060032525205</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>18.65</v>
+        <v>90</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -1771,16 +1771,16 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>51.78397378226776</v>
+        <v>66.90273270880746</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>9.509070762600002</v>
+        <v>33.6386347266467</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>0.9589250626536928</v>
+        <v>0.5606003252520535</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L25" s="2" t="n">
         <v>0</v>
@@ -1789,31 +1789,31 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0.009660062608676001</v>
+        <v>0.9081229621584156</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>8289</v>
+        <v>8093</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>泰藝</t>
+          <t>保銳</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>767.6714930891507</v>
+        <v>769.5892506265369</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>68</v>
+        <v>18.65</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -1824,13 +1824,13 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>56.16594698131369</v>
+        <v>51.78397380531299</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>36.93868404900191</v>
+        <v>9.509070962581204</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>1.267149308915068</v>
+        <v>0.9589250626536928</v>
       </c>
       <c r="K26" s="2" t="n">
         <v>0</v>
@@ -1842,31 +1842,31 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>-0.7984954036322991</v>
+        <v>0.009660062314387799</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>9105</v>
+        <v>8289</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>泰金寶-DR</t>
+          <t>泰藝</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>766.5901563514115</v>
+        <v>767.6714930891507</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>9.529999999999999</v>
+        <v>68</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -1877,13 +1877,13 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>58.05806515481172</v>
+        <v>56.16594698724632</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>51.1560669777375</v>
+        <v>36.93868432484931</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>0.6590156351411459</v>
+        <v>1.267149308915068</v>
       </c>
       <c r="K27" s="2" t="n">
         <v>0</v>
@@ -1895,31 +1895,31 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>-0.1032488904017074</v>
+        <v>-0.798495403689536</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>8050</v>
+        <v>9105</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>廣積</t>
+          <t>泰金寶-DR</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>761.1893660808831</v>
+        <v>766.5901563514115</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>57.7</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -1930,13 +1930,13 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>59.14635035295779</v>
+        <v>58.05806515597874</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>51.22273523185245</v>
+        <v>51.15606710226986</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>0.6189366080883086</v>
+        <v>0.6590156351411459</v>
       </c>
       <c r="K28" s="2" t="n">
         <v>0</v>
@@ -1948,31 +1948,31 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>-0.4312831720554317</v>
+        <v>-0.1032488904341426</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>8472</v>
+        <v>8050</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>夠麻吉</t>
+          <t>廣積</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>760.6060032525205</v>
+        <v>761.1893660808831</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>90</v>
+        <v>57.7</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1983,16 +1983,16 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>66.90273188161098</v>
+        <v>59.14635042923016</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>33.6386344395954</v>
+        <v>51.22273516861638</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>0.5606003252520535</v>
+        <v>0.6189366080883086</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L29" s="2" t="n">
         <v>0</v>
@@ -2001,31 +2001,31 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.9081229670904608</v>
+        <v>-0.4312831724751826</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>8261</v>
+        <v>9904</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>富鼎</t>
+          <t>寶成</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
         <v/>
       </c>
       <c r="D30" s="2" t="n">
-        <v>758.472155059858</v>
+        <v>759.6341737782157</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>173.5</v>
+        <v>26.65</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -2036,16 +2036,16 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>58.98096094605384</v>
+        <v>56.53967831743935</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>36.5528665544884</v>
+        <v>22.09118386215975</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>1.347215505985797</v>
+        <v>0.9634173778215602</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L30" s="2" t="n">
         <v>0</v>
@@ -2054,31 +2054,31 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>-2.906328983063853</v>
+        <v>0.1424122774844594</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
+          <t>rsi_strong, breakout_20d, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>9904</v>
+        <v>8261</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>寶成</t>
+          <t>富鼎</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>744.6341737782157</v>
+        <v>758.472155059858</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>26.65</v>
+        <v>173.5</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -2089,16 +2089,16 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>56.53967810423492</v>
+        <v>58.98096095518385</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>22.09118382481567</v>
+        <v>36.55286669831683</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>0.9634173778215602</v>
+        <v>1.347215505985797</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L31" s="2" t="n">
         <v>0</v>
@@ -2107,31 +2107,31 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.1424122775893979</v>
+        <v>-2.906328983502666</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, breakout_20d, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>8081</v>
+        <v>8996</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>致新</t>
+          <t>高力</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>737.802493723582</v>
+        <v>743.5650969612898</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>283</v>
+        <v>1145</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -2142,49 +2142,49 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>56.58130335777933</v>
+        <v>51.2189153228136</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>27.46160449415379</v>
+        <v>14.32482599366247</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>1.280249372358201</v>
+        <v>0.8565096961289819</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L32" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="M32" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>-2.195606676888061</v>
+        <v>4.089711942645408</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, invest_trust_buy_2d, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>8097</v>
+        <v>8462</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>常珵</t>
+          <t>柏文</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>735.0461943503122</v>
+        <v>738.8404345693505</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>59.8</v>
+        <v>145.5</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -2195,13 +2195,13 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>63.23118683917913</v>
+        <v>61.36327733417813</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>32.01206707489881</v>
+        <v>15.79382974707338</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>1.004619435031228</v>
+        <v>0.8840434569350503</v>
       </c>
       <c r="K33" s="2" t="n">
         <v>1</v>
@@ -2213,31 +2213,31 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>-0.0245751771913982</v>
+        <v>0.7716962495474234</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, bb_squeeze_breakout, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>8996</v>
+        <v>8081</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>高力</t>
+          <t>致新</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>728.5650969612898</v>
+        <v>737.802493723582</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>1145</v>
+        <v>283</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -2248,49 +2248,49 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>51.21891531805601</v>
+        <v>56.58130339362687</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>14.32482578198818</v>
+        <v>27.46160465781798</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>0.8565096961289819</v>
+        <v>1.280249372358201</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L34" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="M34" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>4.089711944553354</v>
+        <v>-2.19560667812825</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, invest_trust_buy_2d, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>8462</v>
+        <v>8097</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>柏文</t>
+          <t>常珵</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>723.8404345693505</v>
+        <v>735.0461943503122</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>145.5</v>
+        <v>59.8</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -2301,13 +2301,13 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>61.36327714834319</v>
+        <v>63.23118680710458</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>15.79382968233157</v>
+        <v>32.01206704788781</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>0.8840434569350503</v>
+        <v>1.004619435031228</v>
       </c>
       <c r="K35" s="2" t="n">
         <v>1</v>
@@ -2319,11 +2319,11 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.7716962502152097</v>
+        <v>-0.0245751772486286</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, bb_squeeze_breakout, mfi_strong</t>
+          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>59.16514049759144</v>
+        <v>59.16514052915869</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>33.08322568489195</v>
+        <v>33.0832257409963</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.7923469301665786</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>0.2829638728420431</v>
+        <v>0.2829638726989492</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>49.92673618322886</v>
+        <v>49.92673620279008</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>24.73824457204842</v>
+        <v>24.7382446428784</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>0.3724149258353246</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>-0.3187602951275028</v>
+        <v>-0.3187602952515223</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2435,21 +2435,21 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>8473</v>
+        <v>8076</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>山林水</t>
+          <t>伍豐</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v/>
       </c>
       <c r="D38" s="2" t="n">
-        <v>715.6752747737261</v>
+        <v>717.3592848436724</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>51.8</v>
+        <v>26.85</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2460,16 +2460,16 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>65.21842135228859</v>
+        <v>60.4820141658874</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>46.2742937176854</v>
+        <v>26.52614041802861</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>0.567527477372602</v>
+        <v>0.7359284843672395</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L38" s="2" t="n">
         <v>0</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>-0.0057997792098394</v>
+        <v>0.1412875694040731</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2488,21 +2488,21 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>8162</v>
+        <v>8473</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>微矽電子-創</t>
+          <t>山林水</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>710.3389990452679</v>
+        <v>715.6752747737261</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>66.90000000000001</v>
+        <v>51.8</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2513,16 +2513,16 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>53.07635221343635</v>
+        <v>65.21842137153347</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>42.43976543026272</v>
+        <v>46.27429391826468</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>0.5338999045267854</v>
+        <v>0.567527477372602</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L39" s="2" t="n">
         <v>0</v>
@@ -2531,31 +2531,31 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-1.623731155841776</v>
+        <v>-0.0057997793624737</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, kd_golden_cross, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>8076</v>
+        <v>9906</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>伍豐</t>
+          <t>欣巴巴</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>702.3592848436724</v>
+        <v>711.8649594822763</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>26.85</v>
+        <v>44.35</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2566,16 +2566,16 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>60.48201410973714</v>
+        <v>67.53965628885631</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>26.52614036792481</v>
+        <v>35.22232649153272</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>0.7359284843672395</v>
+        <v>1.186495948227628</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L40" s="2" t="n">
         <v>0</v>
@@ -2584,31 +2584,31 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>0.1412875695090132</v>
+        <v>1.143799705234902</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>9906</v>
+        <v>8162</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>欣巴巴</t>
+          <t>微矽電子-創</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
         <v/>
       </c>
       <c r="D41" s="2" t="n">
-        <v>696.8649594822763</v>
+        <v>710.3389990452679</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>44.35</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2619,16 +2619,16 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>67.5396562999198</v>
+        <v>53.07635220228205</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>35.2223265768216</v>
+        <v>42.43976555045239</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>1.186495948227628</v>
+        <v>0.5338999045267854</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L41" s="2" t="n">
         <v>0</v>
@@ -2637,31 +2637,31 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>1.143799705826365</v>
+        <v>-1.623731155860844</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, kd_golden_cross, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>8104</v>
+        <v>8429</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>錸寶</t>
+          <t>金麗-KY</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>658.043013258752</v>
+        <v>668.8845254594174</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>38.55</v>
+        <v>6.67</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2672,16 +2672,16 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>50.72746506501572</v>
+        <v>57.8132100866676</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>31.77278177315866</v>
+        <v>28.07988544436479</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>0.3043013258751976</v>
+        <v>0.3884525459417387</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L42" s="2" t="n">
         <v>0</v>
@@ -2690,31 +2690,31 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-0.2651072465997548</v>
+        <v>0.0519451716208445</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>9905</v>
+        <v>8104</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>大華</t>
+          <t>錸寶</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>657.9710804320248</v>
+        <v>658.043013258752</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>20.85</v>
+        <v>38.55</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2725,16 +2725,16 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>51.39369221995201</v>
+        <v>50.72746509859287</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>20.22131909862514</v>
+        <v>31.77278187598197</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>0.7971080432024796</v>
+        <v>0.3043013258751976</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L43" s="2" t="n">
         <v>0</v>
@@ -2743,31 +2743,31 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>0.018570386094846</v>
+        <v>-0.265107246752396</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>8429</v>
+        <v>9905</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>金麗-KY</t>
+          <t>大華</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>653.8845254594174</v>
+        <v>657.9710804320248</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>6.67</v>
+        <v>20.85</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2778,16 +2778,16 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>57.81320995297622</v>
+        <v>51.3936922870185</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>28.0798853611437</v>
+        <v>20.22131897904161</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>0.3884525459417387</v>
+        <v>0.7971080432024796</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L44" s="2" t="n">
         <v>0</v>
@@ -2796,11 +2796,11 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.051945171660912</v>
+        <v>0.0185703860853083</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>47.66946440850688</v>
+        <v>47.66946442405857</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>21.8880836655735</v>
+        <v>21.8880837775817</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.492065525180935</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-2.566693125943666</v>
+        <v>-2.566693126420664</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2884,7 +2884,7 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>52.25772226274382</v>
+        <v>52.2577222444929</v>
       </c>
       <c r="I46" s="2" t="n">
         <v>9.204945459824261</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.0295781514953807</v>
+        <v>0.0295781515049204</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2912,21 +2912,21 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>8374</v>
+        <v>9907</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>羅昇</t>
+          <t>統一實</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>601.5416919995025</v>
+        <v>603.7960207947705</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>90.59999999999999</v>
+        <v>16.7</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2937,16 +2937,16 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>44.7749553739711</v>
+        <v>52.38006271084701</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>25.0378251744584</v>
+        <v>26.53455310154342</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.1541691999502519</v>
+        <v>0.8796020794770439</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L47" s="2" t="n">
         <v>0</v>
@@ -2955,31 +2955,31 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-2.609663077771354</v>
+        <v>0.1260019116609891</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, kd_golden_cross, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>8064</v>
+        <v>8411</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>東捷</t>
+          <t>福貞-KY</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>590.191223605312</v>
+        <v>603.7558794645165</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>134.5</v>
+        <v>12.2</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2990,16 +2990,16 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>49.72336286569056</v>
+        <v>52.58834621160235</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>42.12567421583699</v>
+        <v>30.28018929117312</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>0.5191223605312006</v>
+        <v>0.8755879464516463</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L48" s="2" t="n">
         <v>0</v>
@@ -3008,31 +3008,31 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-4.251331413730117</v>
+        <v>0.0242596861121246</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, cci_momentum</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>9907</v>
+        <v>8374</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>統一實</t>
+          <t>羅昇</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>588.7960207947705</v>
+        <v>601.5416919995025</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>16.7</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,16 +3043,16 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>52.38006261429762</v>
+        <v>44.77495540076246</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>26.53455309159187</v>
+        <v>25.03782534308142</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>0.8796020794770439</v>
+        <v>0.1541691999502519</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L49" s="2" t="n">
         <v>0</v>
@@ -3061,31 +3061,31 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.1260019116991479</v>
+        <v>-2.609663078343734</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, kd_golden_cross, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>8411</v>
+        <v>9911</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>福貞-KY</t>
+          <t>櫻花</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>588.7558794645165</v>
+        <v>601.3782710001745</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>12.2</v>
+        <v>84.3</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,16 +3096,16 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>52.58834632342011</v>
+        <v>56.07408032624189</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>30.28018829686007</v>
+        <v>19.45392506711162</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0.8755879464516463</v>
+        <v>0.6378271000174536</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="L50" s="2" t="n">
         <v>0</v>
@@ -3114,31 +3114,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>0.0242596860739644</v>
+        <v>0.3121549554797315</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, cci_momentum</t>
+          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>9930</v>
+        <v>8064</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>中聯資源</t>
+          <t>東捷</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>587.7136812955025</v>
+        <v>590.191223605312</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>69.5</v>
+        <v>134.5</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,16 +3149,16 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>53.94989912164106</v>
+        <v>49.72336287808143</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>15.33408484321537</v>
+        <v>42.12567409193138</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.7713681295502544</v>
+        <v>0.5191223605312006</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L51" s="2" t="n">
         <v>0</v>
@@ -3167,31 +3167,31 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.1143908996178223</v>
+        <v>-4.251331413806435</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>9911</v>
+        <v>8422</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>櫻花</t>
+          <t>可寧衛*</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>586.3782710001745</v>
+        <v>588.9959577563864</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>84.3</v>
+        <v>29</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3202,49 +3202,49 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>56.07408028108178</v>
+        <v>55.67889577476007</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>19.45392513399611</v>
+        <v>18.18863198646347</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.6378271000174536</v>
+        <v>0.8995957756386314</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L52" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M52" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>0.3121549556514467</v>
+        <v>0.3261087174887492</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>8271</v>
+        <v>9930</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>宇瞻</t>
+          <t>中聯資源</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>583.4569476677641</v>
+        <v>587.7136812955025</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>202.5</v>
+        <v>69.5</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,16 +3255,16 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>40.62117169987642</v>
+        <v>53.94989910992317</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>25.7221280206245</v>
+        <v>15.33408486577226</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.8456947667764119</v>
+        <v>0.7713681295502544</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L53" s="2" t="n">
         <v>0</v>
@@ -3273,31 +3273,31 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>-6.371842913966106</v>
+        <v>0.1143908996559835</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>8383</v>
+        <v>8067</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>千附</t>
+          <t>志旭</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>583.050940330603</v>
+        <v>587.0347993688246</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>58.7</v>
+        <v>13</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,16 +3308,16 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>49.65017347857378</v>
+        <v>51.11994057162706</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>16.70310544685576</v>
+        <v>7.718372432977032</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.3050940330603038</v>
+        <v>2.20347993688246</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L54" s="2" t="n">
         <v>0</v>
@@ -3326,31 +3326,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>-0.3369058031935129</v>
+        <v>-0.0896229609264925</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross, obv_uptrend</t>
+          <t>above_ema60, volume_break, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>8422</v>
+        <v>8271</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>可寧衛*</t>
+          <t>宇瞻</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>573.9959577563864</v>
+        <v>583.4569476677641</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>29</v>
+        <v>202.5</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,49 +3361,49 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>55.67889548395547</v>
+        <v>40.62117170580096</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>18.18863183877251</v>
+        <v>25.7221280262651</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.8995957756386314</v>
+        <v>0.8456947667764119</v>
       </c>
       <c r="K55" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L55" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M55" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.3261087181427229</v>
+        <v>-6.371842914156865</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>8463</v>
+        <v>8383</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>潤泰材</t>
+          <t>千附</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>572.9133535560627</v>
+        <v>583.050940330603</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>22.3</v>
+        <v>58.7</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,16 +3414,16 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>55.9016326870443</v>
+        <v>49.65017348983083</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>12.90760947582078</v>
+        <v>16.70310557785773</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>0.7913353556062663</v>
+        <v>0.3050940330603038</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.0990193562676399</v>
+        <v>-0.3369058034701633</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>8067</v>
+        <v>8463</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>志旭</t>
+          <t>潤泰材</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>572.0347993688246</v>
+        <v>572.9133535560627</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>13</v>
+        <v>22.3</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,13 +3467,13 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>51.11994053400343</v>
+        <v>55.90163272935447</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>7.718372405816232</v>
+        <v>12.90760947924843</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>2.20347993688246</v>
+        <v>0.7913353556062663</v>
       </c>
       <c r="K57" s="2" t="n">
         <v>0</v>
@@ -3485,11 +3485,11 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-0.08962296076431669</v>
+        <v>0.0990193562008649</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, volume_break, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
@@ -3506,7 +3506,7 @@
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>556.7840229576329</v>
+        <v>571.7840229576329</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>48.5</v>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>51.59358904442688</v>
+        <v>51.59358908053441</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>6.451353797287808</v>
+        <v>6.451353768248037</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>0.1784022957632988</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.331522822459511</v>
+        <v>0.3315228218871322</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3548,21 +3548,21 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>8049</v>
+        <v>9103</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>晶采</t>
+          <t>美德醫療-DR</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>553.3941757174393</v>
+        <v>554.783875385485</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>26.3</v>
+        <v>5.62</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,16 +3573,16 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>48.13639455923172</v>
+        <v>55.90472982865833</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>22.04055248915984</v>
+        <v>41.47900168162743</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.3394175717439293</v>
+        <v>0.4783875385484964</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.1336733893415811</v>
+        <v>0.0248687093144894</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>9103</v>
+        <v>8049</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>美德醫療-DR</t>
+          <t>晶采</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>539.783875385485</v>
+        <v>553.3941757174393</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>5.62</v>
+        <v>26.3</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,16 +3626,16 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>55.90472977536304</v>
+        <v>48.13639458206295</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>41.47900163630806</v>
+        <v>22.04055251216093</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>0.4783875385484964</v>
+        <v>0.3394175717439293</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.0248687093602802</v>
+        <v>-0.1336733894274402</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>8201</v>
+        <v>9912</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>無敵</t>
+          <t>偉聯</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>525.2014511148109</v>
+        <v>532.5016519108142</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>13.25</v>
+        <v>12.5</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,13 +3679,13 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>49.73681354705163</v>
+        <v>49.74383526098858</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>24.27691278897154</v>
+        <v>18.71296263210416</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.52014511148108</v>
+        <v>0.2501651910814164</v>
       </c>
       <c r="K61" s="2" t="n">
         <v>0</v>
@@ -3697,31 +3697,31 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-0.0534954650708059</v>
+        <v>0.0040206199443547</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>9912</v>
+        <v>8443</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>偉聯</t>
+          <t>阿瘦</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>517.5016519108142</v>
+        <v>526.4219064931926</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>12.5</v>
+        <v>11.4</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3732,13 +3732,13 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>49.7438355546564</v>
+        <v>48.28717672865851</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>18.71296262675999</v>
+        <v>60.11586989590077</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>0.2501651910814164</v>
+        <v>1.642190649319267</v>
       </c>
       <c r="K62" s="2" t="n">
         <v>0</v>
@@ -3750,31 +3750,31 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>0.0040206198966559</v>
+        <v>0.0367381808265993</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>8114</v>
+        <v>8201</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>振樺電</t>
+          <t>無敵</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>512.8460418580135</v>
+        <v>525.2014511148109</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>210.5</v>
+        <v>13.25</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,13 +3785,13 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>44.47379711765936</v>
+        <v>49.7368135979366</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>32.22285001013758</v>
+        <v>24.27691283343341</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>0.7846041858013412</v>
+        <v>0.52014511148108</v>
       </c>
       <c r="K63" s="2" t="n">
         <v>0</v>
@@ -3803,31 +3803,31 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-6.966905046601398</v>
+        <v>-0.0534954651662034</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>8443</v>
+        <v>8114</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>阿瘦</t>
+          <t>振樺電</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>511.4219064931926</v>
+        <v>512.8460418580135</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>11.4</v>
+        <v>210.5</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,13 +3838,13 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>48.28717672865851</v>
+        <v>44.47379714428499</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>60.11586992781709</v>
+        <v>32.22285005636553</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>1.642190649319267</v>
+        <v>0.7846041858013412</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0</v>
@@ -3856,11 +3856,11 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>0.0367381808170599</v>
+        <v>-6.966905048318544</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, cci_momentum, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>45.77996731171856</v>
+        <v>45.77996734763395</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>36.44195539376538</v>
+        <v>36.44195539917453</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.5548500708933531</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-2.118122894618721</v>
+        <v>-2.118122893721997</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>51.86939471282546</v>
+        <v>51.86939428163027</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>24.93714223611338</v>
+        <v>24.93714231181037</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>0.3524711159358183</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.00415995058068</v>
+        <v>0.0041599507619372</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>53.58872082657346</v>
+        <v>53.58872083318042</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>14.61789929360733</v>
+        <v>14.61789929360734</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.4393309280527326</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-0.120983541271725</v>
+        <v>-0.1209835413480449</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>46.21250486130602</v>
+        <v>46.21250481306858</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>30.93064125847625</v>
+        <v>30.93064129097599</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>0.6532696083181547</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-6.632268163549728</v>
+        <v>-6.632268164217512</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>37.78092686953038</v>
+        <v>37.78092689087535</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>18.37027267105078</v>
+        <v>18.37027278127145</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.3716854036942976</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-1.043482102798902</v>
+        <v>-1.04348210305648</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4131,21 +4131,21 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>8110</v>
+        <v>8404</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>華東</t>
+          <t>百和興業-KY</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>460.1333725472123</v>
+        <v>470.4089647861393</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>54.8</v>
+        <v>17.35</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,16 +4156,16 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>50.72454355420085</v>
+        <v>53.78836849047874</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>16.68065012847181</v>
+        <v>18.02091619808385</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.5133372547212286</v>
+        <v>0.5408964786139359</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L70" s="2" t="n">
         <v>0</v>
@@ -4174,31 +4174,31 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-0.7263441315923429</v>
+        <v>0.1145656714590461</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>8404</v>
+        <v>8110</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>百和興業-KY</t>
+          <t>華東</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>455.4089647861393</v>
+        <v>460.1333725472123</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>17.35</v>
+        <v>54.8</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,16 +4209,16 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>53.78836828526399</v>
+        <v>50.72454356190513</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>18.02091614003154</v>
+        <v>16.6806501284718</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.5408964786139359</v>
+        <v>0.5133372547212286</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L71" s="2" t="n">
         <v>0</v>
@@ -4227,31 +4227,31 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.1145656715544448</v>
+        <v>-0.7263441316400348</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>8367</v>
+        <v>8087</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>建新國際</t>
+          <t>華鎂鑫</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>453.2556408090207</v>
+        <v>456.4753359757303</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>40.35</v>
+        <v>33.85</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,13 +4262,13 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>33.72133049250023</v>
+        <v>47.10298831054512</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>26.91791568739532</v>
+        <v>25.34585106319381</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.3255640809020665</v>
+        <v>0.6475335975730353</v>
       </c>
       <c r="K72" s="2" t="n">
         <v>0</v>
@@ -4280,31 +4280,31 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>0.0010237060819854</v>
+        <v>0.1108378871911429</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>8087</v>
+        <v>8367</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>華鎂鑫</t>
+          <t>建新國際</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>441.4753359757303</v>
+        <v>453.2556408090207</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>33.85</v>
+        <v>40.35</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -4315,13 +4315,13 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>47.10298815793712</v>
+        <v>33.72133061503209</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>25.34585106398508</v>
+        <v>26.9179157372861</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>0.6475335975730353</v>
+        <v>0.3255640809020665</v>
       </c>
       <c r="K73" s="2" t="n">
         <v>0</v>
@@ -4333,11 +4333,11 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>0.1108378877253689</v>
+        <v>0.001023705862569</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
@@ -4354,7 +4354,7 @@
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>438.179362691882</v>
+        <v>453.179362691882</v>
       </c>
       <c r="E74" s="2" t="n">
         <v>3.5</v>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>58.48918598956655</v>
+        <v>58.48919028148045</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>19.59257004253818</v>
+        <v>19.5925701496666</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0.3179362691882041</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.0431969377247836</v>
+        <v>0.0431969365513975</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>42.28341637464622</v>
+        <v>42.28341639217842</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>28.21234762369997</v>
+        <v>28.21234773415222</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>0.6249332678672165</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-7.205170339108433</v>
+        <v>-7.205170340062433</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>45.92304281516252</v>
+        <v>45.923042756091</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>34.93077077751785</v>
+        <v>34.93077083234853</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.3124061644474037</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.4077304017607541</v>
+        <v>-0.4077304015318024</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>42.46379780901534</v>
+        <v>42.46379784862845</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>28.95113263449281</v>
+        <v>28.95113266033416</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.2995683010195427</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-1.93146179471104</v>
+        <v>-1.931461794777813</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>42.41236080512724</v>
+        <v>42.41236087442611</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>23.27640456207093</v>
+        <v>23.27640463199956</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.1760739824123672</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.7362139110333903</v>
+        <v>-0.7362139113768229</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4608,21 +4608,21 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>8466</v>
+        <v>9802</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>美吉吉-KY</t>
+          <t>鈺齊-KY</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>422.5496902017919</v>
+        <v>427.0379700060529</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>16.1</v>
+        <v>79.2</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4633,16 +4633,16 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>52.9083963262533</v>
+        <v>52.98068382920669</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>26.74835257080058</v>
+        <v>16.30299771596123</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>0.2549690201791838</v>
+        <v>0.703797000605293</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L79" s="2" t="n">
         <v>0</v>
@@ -4651,31 +4651,31 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>0.0925971534325971</v>
+        <v>0.4327854135939614</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>8155</v>
+        <v>8466</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>博智</t>
+          <t>美吉吉-KY</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>421.8322726179034</v>
+        <v>422.5496902017919</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>351.5</v>
+        <v>16.1</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4686,16 +4686,16 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>36.85921105904809</v>
+        <v>52.90839634204371</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>24.35859796766492</v>
+        <v>26.74835245324017</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>0.6832272617903479</v>
+        <v>0.2549690201791838</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L80" s="2" t="n">
         <v>0</v>
@@ -4704,31 +4704,31 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-7.730672001978188</v>
+        <v>0.0925971532990421</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>9802</v>
+        <v>8155</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>鈺齊-KY</t>
+          <t>博智</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>412.0379700060529</v>
+        <v>421.8322726179034</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>79.2</v>
+        <v>351.5</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,16 +4739,16 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>52.98068365086494</v>
+        <v>36.85921108043143</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>16.30299769633535</v>
+        <v>24.35859843311814</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>0.703797000605293</v>
+        <v>0.6832272617903479</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L81" s="2" t="n">
         <v>0</v>
@@ -4757,11 +4757,11 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.4327854143571349</v>
+        <v>-7.730672003695382</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
@@ -4792,7 +4792,7 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>47.30843009632142</v>
+        <v>47.30843021698072</v>
       </c>
       <c r="I82" s="2" t="n">
         <v>10.92277531091451</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>0.0233411798506212</v>
+        <v>0.0233411797933815</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>47.90254991091283</v>
+        <v>47.90254991151587</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>18.69520457335457</v>
+        <v>18.69520464200195</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.5985946876021407</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-64.72739800830813</v>
+        <v>-64.72739800992943</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>42.08609022080457</v>
+        <v>42.08609025432503</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>11.63772003568072</v>
+        <v>11.6377201961175</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>0.4076065730124188</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.5605119668881091</v>
+        <v>-0.5605119674223225</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4926,21 +4926,21 @@
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>8111</v>
+        <v>9908</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>立碁</t>
+          <t>大台北</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>379.6022293338205</v>
+        <v>384.9653099326629</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>55.6</v>
+        <v>29.4</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,13 +4951,13 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>32.69104026113976</v>
+        <v>51.72114706388812</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>22.89424982168907</v>
+        <v>12.69780630702978</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.4602229333820502</v>
+        <v>0.996530993266296</v>
       </c>
       <c r="K85" s="2" t="n">
         <v>0</v>
@@ -4969,31 +4969,31 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-0.951020528552854</v>
+        <v>0.0468871865560187</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>9908</v>
+        <v>8080</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>大台北</t>
+          <t>永利聯合</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>369.9653099326629</v>
+        <v>383.2253651076522</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>29.4</v>
+        <v>28</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5004,16 +5004,16 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>51.72114698608598</v>
+        <v>48.07376366785177</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>12.69780630702978</v>
+        <v>36.00045910955024</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.996530993266296</v>
+        <v>1.822536510765225</v>
       </c>
       <c r="K86" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L86" s="2" t="n">
         <v>0</v>
@@ -5022,31 +5022,31 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>0.0468871865846345</v>
+        <v>0.07411339006789799</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>8080</v>
+        <v>8111</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>永利聯合</t>
+          <t>立碁</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>368.2253651076522</v>
+        <v>379.6022293338205</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>28</v>
+        <v>55.6</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,16 +5057,16 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>48.07376360915477</v>
+        <v>32.6910403529488</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>36.00045903209691</v>
+        <v>22.89425015809781</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>1.822536510765225</v>
+        <v>0.4602229333820502</v>
       </c>
       <c r="K87" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L87" s="2" t="n">
         <v>0</v>
@@ -5075,11 +5075,11 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.0741133902682302</v>
+        <v>-0.9510205292110968</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, stronger_than_market</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>46.53403068465418</v>
+        <v>46.53403056053281</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>12.13378868062859</v>
+        <v>12.13378869306298</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>0.9421855080631028</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.0392611625310781</v>
+        <v>0.039261162616932</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5163,16 +5163,16 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>53.71905015625882</v>
+        <v>53.71904893706057</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>19.23218496319492</v>
+        <v>19.23218395533451</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.9081772784019976</v>
       </c>
       <c r="K89" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L89" s="2" t="n">
         <v>0</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>0.0722338337470818</v>
+        <v>0.0722338368188729</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>44.75464605438582</v>
+        <v>44.7546460834613</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>17.93556239042444</v>
+        <v>17.93556255581226</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.6601147613173324</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-0.4258020730822641</v>
+        <v>-0.4258020731776635</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5244,21 +5244,21 @@
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>8103</v>
+        <v>8423</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>瀚荃</t>
+          <t>保綠-KY</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>334.4677188704329</v>
+        <v>339.842305985859</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>97</v>
+        <v>17.75</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,16 +5269,16 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>41.79376322767571</v>
+        <v>47.4095852222886</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>18.17697526456949</v>
+        <v>11.60409782324896</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>0.4467718870432877</v>
+        <v>0.4842305985858986</v>
       </c>
       <c r="K91" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L91" s="2" t="n">
         <v>0</v>
@@ -5287,31 +5287,31 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-1.352741767382678</v>
+        <v>0.024609051342882</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>8423</v>
+        <v>8103</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>保綠-KY</t>
+          <t>瀚荃</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>324.842305985859</v>
+        <v>334.4677188704329</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>17.75</v>
+        <v>97</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5322,16 +5322,16 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>47.40958550120996</v>
+        <v>41.7937632565839</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>11.60409787385631</v>
+        <v>18.17697521086277</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>0.4842305985858986</v>
+        <v>0.4467718870432877</v>
       </c>
       <c r="K92" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L92" s="2" t="n">
         <v>0</v>
@@ -5340,11 +5340,11 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>0.0246090513142629</v>
+        <v>-1.352741767595231</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
         </is>
       </c>
     </row>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>42.75794922279159</v>
+        <v>42.75794934959161</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>22.7986842378808</v>
+        <v>22.79868440123157</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>0.2735824963286599</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-1.066909552125648</v>
+        <v>-1.066909553499369</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>50.98067546119956</v>
+        <v>50.98067576399289</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>28.16007219567909</v>
+        <v>28.16007235048496</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>0.8086031470403593</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0.1256219017229988</v>
+        <v>0.1256219007499455</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>34.3969982636208</v>
+        <v>34.39699830292857</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>21.33679329465758</v>
+        <v>21.3367934174281</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>1.188114946447997</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.07490399365169551</v>
+        <v>-0.07490399383294739</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>37.08970576359114</v>
+        <v>37.08970580840941</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>21.45134564636817</v>
+        <v>21.45134583155563</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.6381684234567122</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-3.954902896032969</v>
+        <v>-3.954902896738932</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>43.21812319524983</v>
+        <v>43.21812349811794</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>16.7342832518673</v>
+        <v>16.73428336340897</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.7255768677022472</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-0.2429466736837537</v>
+        <v>-0.2429466741416643</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>45.49957029330114</v>
+        <v>45.49957033547269</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>14.81211467739793</v>
+        <v>14.81211468666623</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.4348643378776876</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.025258760578283</v>
+        <v>-0.0252587607404638</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>44.73138628605845</v>
+        <v>44.73138629865668</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>13.60305774743609</v>
+        <v>13.6030577323142</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.4057803295100132</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.0075708714754372</v>
+        <v>-0.0075708715135971</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>35.029200638275</v>
+        <v>35.02920064998307</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>23.58001525850659</v>
+        <v>23.58001522265481</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.2550971449927526</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.4131822047494544</v>
+        <v>-0.4131822047589922</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>47.92742897991698</v>
+        <v>47.92742899012291</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>15.94559741118474</v>
+        <v>15.94559757279222</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.6438904690793427</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-3.805548349631437</v>
+        <v>-3.805548349726837</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>37.6382129477252</v>
+        <v>37.63821297952412</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>23.74587731558962</v>
+        <v>23.74587732990783</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>0.6285205161781295</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.1048843206794437</v>
+        <v>-0.104884320135679</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>44.45762343521315</v>
+        <v>44.45762344316263</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>16.475311015498</v>
+        <v>16.47531098699172</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.5562899973700359</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.0894852295936342</v>
+        <v>-0.08948522984166909</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>44.1167716699802</v>
+        <v>44.11677167809043</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>11.29237361136654</v>
+        <v>11.29237378574422</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>0.694552116399459</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.8067620068746564</v>
+        <v>-0.8067620070082204</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>51.74212264045482</v>
+        <v>51.74212273377388</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>20.19032251909788</v>
+        <v>20.19032262434558</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>1.070145843781503</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.0371667563839681</v>
+        <v>-0.0371667565556832</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>40.09429923034781</v>
+        <v>40.09429927271883</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>15.25094376575684</v>
+        <v>15.25094402865202</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>0.4514640066352793</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-1.191043859393149</v>
+        <v>-1.191043859622107</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6103,7 +6103,7 @@
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>236.2991654296167</v>
+        <v>251.2991654296167</v>
       </c>
       <c r="E107" s="2" t="n">
         <v>40.2</v>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>33.7696645492039</v>
+        <v>33.76966461303857</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>26.40921108874634</v>
+        <v>26.40921104120241</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>0.629916542961673</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>0.4469937118833313</v>
+        <v>0.4469937114063484</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6145,21 +6145,21 @@
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>8059</v>
+        <v>8478</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>凱碩</t>
+          <t>東哥遊艇</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>219.5208461091036</v>
+        <v>230.2673075781701</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>18.15</v>
+        <v>152.5</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -6170,13 +6170,13 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>41.25942474094335</v>
+        <v>42.64756283409948</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>18.3082526134114</v>
+        <v>19.8245939185917</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>0.4520846109103542</v>
+        <v>1.026730757817008</v>
       </c>
       <c r="K108" s="2" t="n">
         <v>0</v>
@@ -6188,31 +6188,31 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.174115715675983</v>
+        <v>0.4937160912076102</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>8478</v>
+        <v>8059</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>東哥遊艇</t>
+          <t>凱碩</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>215.2673075781701</v>
+        <v>219.5208461091036</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>152.5</v>
+        <v>18.15</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,13 +6223,13 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>42.64756274391355</v>
+        <v>41.25942482059413</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>19.82459377726554</v>
+        <v>18.3082526504627</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>1.026730757817008</v>
+        <v>0.4520846109103542</v>
       </c>
       <c r="K109" s="2" t="n">
         <v>0</v>
@@ -6241,11 +6241,11 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.4937160925431849</v>
+        <v>-0.1741157158953962</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>7.411176855991869</v>
+        <v>7.411176859887959</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>23.61214963983392</v>
+        <v>23.612149573302</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.0065554287439043</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-7.634066825046457</v>
+        <v>-7.634066826286626</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>46.00471770145328</v>
+        <v>46.00471790330297</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>17.32165907043329</v>
+        <v>17.32165911024971</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.2362547491860861</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.1301573596983648</v>
+        <v>-0.130157359860538</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>48.35858342107961</v>
+        <v>48.35858345788763</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>29.16332567572406</v>
+        <v>29.16332569447108</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.4935736032007342</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.0941291166428993</v>
+        <v>0.0941291163948666</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>31.56563693765075</v>
+        <v>31.56563691930494</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>17.1118449053259</v>
+        <v>17.11184491743529</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.554187232445371</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.6887884702115676</v>
+        <v>-0.688788470135254</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>40.85024180278165</v>
+        <v>40.85024194996884</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>18.5645773588915</v>
+        <v>18.5645770717894</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>1.93781621081415</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.0168761339509377</v>
+        <v>-0.0168761342943702</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>

</xml_diff>